<commit_message>
chore(client-data): 🔧 Sync brand overlay from canonical client-data
Regenerated from client-data @ 6eaac6f via scripts/sync.sh client-data.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/companies/amaris/amaris-client-data-overview.xlsx
+++ b/companies/amaris/amaris-client-data-overview.xlsx
@@ -32,53 +32,53 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Century Gothic"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00272674"/>
       <sz val="18"/>
     </font>
     <font>
-      <name val="Century Gothic"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="004182ff"/>
       <sz val="12"/>
     </font>
     <font>
-      <name val="Century Gothic"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Century Gothic"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00272674"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Century Gothic"/>
+      <name val="Calibri"/>
       <color rgb="00494951"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Century Gothic"/>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="006c757d"/>
       <sz val="8"/>
     </font>
     <font>
-      <name val="Century Gothic"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
-      <name val="Century Gothic"/>
+      <name val="Calibri"/>
       <color rgb="00494951"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Century Gothic"/>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00272674"/>
       <sz val="9"/>
@@ -680,7 +680,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>producer</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>83</t>
         </is>
       </c>
     </row>
@@ -1289,12 +1289,12 @@
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t>.build-history/~$amaris-client-data-overview.xlsx</t>
+          <t>amaris-client-data-overview.xlsx</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>.build-history</t>
+          <t>root</t>
         </is>
       </c>
       <c r="C9" s="9" t="inlineStr">
@@ -1304,12 +1304,12 @@
       </c>
       <c r="D9" s="9" t="inlineStr">
         <is>
-          <t>0.2 KB</t>
+          <t>18.2 KB</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Build artifact / history record</t>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="D11" s="9" t="inlineStr">
         <is>
-          <t>7.1 KB</t>
+          <t>8.5 KB</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -2168,7 +2168,7 @@
       </c>
       <c r="D41" s="9" t="inlineStr">
         <is>
-          <t>3.3 KB</t>
+          <t>4.0 KB</t>
         </is>
       </c>
       <c r="E41" s="10" t="inlineStr">
@@ -3491,7 +3491,7 @@
       </c>
       <c r="D90" s="11" t="inlineStr">
         <is>
-          <t>2.6 KB</t>
+          <t>3.0 KB</t>
         </is>
       </c>
       <c r="E90" s="12" t="inlineStr">
@@ -3523,7 +3523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3853,116 +3853,143 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
+          <t>Backgroundalt</t>
+        </is>
+      </c>
+      <c r="C15" s="14" t="inlineStr">
+        <is>
+          <t>#F8F9FA</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="inlineStr">
+        <is>
+          <t>rgb(248, 249, 250)</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>Additional brand color</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   </t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
           <t>Sectorcolors / Lifesciences</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>#7DDEB8</t>
         </is>
       </c>
-      <c r="D15" s="14" t="inlineStr">
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>rgb(125, 222, 184)</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E16" s="17" t="inlineStr">
         <is>
           <t>Sectorcolors sector / variant</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="26" t="inlineStr">
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>Sectorcolors / Engineering</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>#B880FF</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D17" s="14" t="inlineStr">
         <is>
           <t>rgb(184, 128, 255)</t>
         </is>
       </c>
-      <c r="E16" s="17" t="inlineStr">
+      <c r="E17" s="15" t="inlineStr">
         <is>
           <t>Sectorcolors sector / variant</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="24" t="inlineStr">
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
         <is>
           <t>Sectorcolors / Telecom</t>
         </is>
       </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>#FFDD77</t>
         </is>
       </c>
-      <c r="D17" s="14" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>rgb(255, 221, 119)</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>Sectorcolors sector / variant</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="18" t="inlineStr">
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="18" t="inlineStr">
         <is>
           <t xml:space="preserve">   </t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Sectorcolors / Digital</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>#4182FF</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D19" s="14" t="inlineStr">
         <is>
           <t>rgb(65, 130, 255)</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="E19" s="15" t="inlineStr">
         <is>
           <t>Sectorcolors sector / variant</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="8" customHeight="1"/>
-    <row r="20">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="20" ht="8" customHeight="1"/>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Amaris Consulting  ·  Confidential — Not for distribution</t>
         </is>
@@ -3970,7 +3997,7 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A20:F20"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3983,7 +4010,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4057,22 +4084,22 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>General Sans</t>
+          <t>Century Gothic</t>
         </is>
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>700</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Semibold</t>
+          <t>Bold</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>Century Gothic</t>
+          <t>Calibri</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr">
@@ -4089,7 +4116,7 @@
       </c>
       <c r="B6" s="11" t="inlineStr">
         <is>
-          <t>General Sans</t>
+          <t>Century Gothic</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -4104,7 +4131,7 @@
       </c>
       <c r="E6" s="11" t="inlineStr">
         <is>
-          <t>Century Gothic</t>
+          <t>Calibri</t>
         </is>
       </c>
       <c r="F6" s="12" t="inlineStr">
@@ -4121,22 +4148,22 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>General Sans</t>
+          <t>Century Gothic</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>500</t>
+          <t>700</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Bold</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>Century Gothic</t>
+          <t>Calibri</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
@@ -4208,66 +4235,42 @@
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Web</t>
+          <t>Embed</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>fonts/web/</t>
+          <t>fonts/otf/ (+ fonts/ttf/) — General Sans, OFL, embeddable</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Css</t>
+          <t>Web</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>fonts/web/general-sans.css</t>
+          <t>fonts/web/ — General Sans woff2</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Otf</t>
+          <t>Note</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>fonts/otf/</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Variable</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t>fonts/ttf/GeneralSans-Variable.ttf</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>License</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>Fontshare Free For Personal &amp; Commercial Use</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="8" customHeight="1"/>
-    <row r="19">
-      <c r="A19" s="7" t="inlineStr">
+          <t>Century Gothic (the named brand face) is a licensed system/Office font — present on the client's own machines but NOT redistributable, so it cannot be embedded server-side. General Sans is the OFL embeddable substitute: server-rendered deliverables embed it (self-contained everywhere); when the client edits on a licensed machine the named Century Gothic still resolves; web uses the General Sans woff2 set.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="8" customHeight="1"/>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>Amaris Consulting  ·  Confidential — Not for distribution</t>
         </is>
@@ -4275,8 +4278,8 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A17:F17"/>
     <mergeCell ref="A10:F10"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>